<commit_message>
Added new RDF data schemes and visual schemes for environment-table15-16, and fixed XLSX spreadsheets for environment-table15-16
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/environment-table15.xlsx
+++ b/sources/table_normalization/xlsx/environment-table15.xlsx
@@ -200,7 +200,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -222,6 +222,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -372,7 +378,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -462,9 +468,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -489,30 +492,32 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -819,7 +824,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1668,70 +1673,70 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:25" s="2" customFormat="1" ht="20">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="46" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1"/>
     </row>
     <row r="4" spans="1:25" s="3" customFormat="1" ht="18">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
-      <c r="H4" s="52"/>
-      <c r="I4" s="52"/>
-      <c r="J4" s="52"/>
-      <c r="K4" s="53"/>
-      <c r="L4" s="54"/>
-      <c r="M4" s="55"/>
-      <c r="N4" s="56"/>
-      <c r="O4" s="52"/>
-      <c r="P4" s="55"/>
-      <c r="Q4" s="55"/>
-      <c r="R4" s="57"/>
-      <c r="S4" s="57"/>
-      <c r="T4" s="52"/>
-      <c r="U4" s="52"/>
-      <c r="V4" s="52"/>
-      <c r="W4" s="57" t="s">
+      <c r="B4" s="49"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="49"/>
+      <c r="F4" s="49"/>
+      <c r="G4" s="49"/>
+      <c r="H4" s="49"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="49"/>
+      <c r="K4" s="55"/>
+      <c r="L4" s="56"/>
+      <c r="M4" s="57"/>
+      <c r="N4" s="58"/>
+      <c r="O4" s="49"/>
+      <c r="P4" s="57"/>
+      <c r="Q4" s="57"/>
+      <c r="R4" s="59"/>
+      <c r="S4" s="59"/>
+      <c r="T4" s="49"/>
+      <c r="U4" s="49"/>
+      <c r="V4" s="49"/>
+      <c r="W4" s="59" t="s">
         <v>2</v>
       </c>
-      <c r="X4" s="57"/>
-      <c r="Y4" s="52"/>
+      <c r="X4" s="59"/>
+      <c r="Y4" s="49"/>
     </row>
     <row r="5" spans="1:25">
-      <c r="A5" s="49" t="s">
+      <c r="A5" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="58"/>
-      <c r="C5" s="59"/>
-      <c r="D5" s="59"/>
-      <c r="E5" s="60"/>
-      <c r="F5" s="61"/>
-      <c r="G5" s="59"/>
-      <c r="H5" s="59"/>
-      <c r="I5" s="59"/>
-      <c r="J5" s="59"/>
-      <c r="K5" s="59"/>
-      <c r="L5" s="59"/>
-      <c r="M5" s="59"/>
-      <c r="N5" s="59"/>
-      <c r="O5" s="59"/>
-      <c r="P5" s="62"/>
-      <c r="Q5" s="62"/>
-      <c r="R5" s="59"/>
-      <c r="S5" s="59"/>
-      <c r="T5" s="63"/>
-      <c r="U5" s="63"/>
-      <c r="V5" s="63"/>
-      <c r="W5" s="63"/>
-      <c r="X5" s="63"/>
-      <c r="Y5" s="63"/>
+      <c r="B5" s="51"/>
+      <c r="C5" s="52"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="53"/>
+      <c r="F5" s="54"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="52"/>
+      <c r="K5" s="52"/>
+      <c r="L5" s="52"/>
+      <c r="M5" s="52"/>
+      <c r="N5" s="52"/>
+      <c r="O5" s="52"/>
+      <c r="P5" s="60"/>
+      <c r="Q5" s="60"/>
+      <c r="R5" s="52"/>
+      <c r="S5" s="52"/>
+      <c r="T5" s="61"/>
+      <c r="U5" s="61"/>
+      <c r="V5" s="61"/>
+      <c r="W5" s="61"/>
+      <c r="X5" s="61"/>
+      <c r="Y5" s="61"/>
     </row>
     <row r="6" spans="1:25">
       <c r="A6" s="50"/>
@@ -2732,111 +2737,111 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:25" s="43" customFormat="1" ht="21" customHeight="1">
-      <c r="A19" s="37" t="s">
+    <row r="19" spans="1:25" s="42" customFormat="1" ht="21" customHeight="1">
+      <c r="A19" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="38">
+      <c r="B19" s="37">
         <v>3480.3</v>
       </c>
-      <c r="C19" s="38">
+      <c r="C19" s="37">
         <v>3315.1</v>
       </c>
-      <c r="D19" s="38">
+      <c r="D19" s="37">
         <v>3207.1</v>
       </c>
-      <c r="E19" s="39">
+      <c r="E19" s="38">
         <v>3242.4</v>
       </c>
-      <c r="F19" s="39">
+      <c r="F19" s="38">
         <v>2928.3</v>
       </c>
-      <c r="G19" s="39">
+      <c r="G19" s="38">
         <v>2827.7</v>
       </c>
-      <c r="H19" s="39">
+      <c r="H19" s="38">
         <v>2842.4</v>
       </c>
-      <c r="I19" s="39">
+      <c r="I19" s="38">
         <v>2709.6</v>
       </c>
-      <c r="J19" s="39">
+      <c r="J19" s="38">
         <v>2716.6</v>
       </c>
-      <c r="K19" s="40">
+      <c r="K19" s="39">
         <v>2635.9690000000001</v>
       </c>
-      <c r="L19" s="41">
+      <c r="L19" s="40">
         <v>2659.7</v>
       </c>
-      <c r="M19" s="41">
+      <c r="M19" s="40">
         <v>2656.8</v>
       </c>
-      <c r="N19" s="41">
+      <c r="N19" s="40">
         <v>2714.7</v>
       </c>
-      <c r="O19" s="41">
+      <c r="O19" s="40">
         <v>2622.4419999999996</v>
       </c>
-      <c r="P19" s="41">
+      <c r="P19" s="40">
         <v>2732.7120000000004</v>
       </c>
-      <c r="Q19" s="41">
+      <c r="Q19" s="40">
         <v>2791.7809999999995</v>
       </c>
-      <c r="R19" s="41">
+      <c r="R19" s="40">
         <v>2854.944</v>
       </c>
-      <c r="S19" s="41">
+      <c r="S19" s="40">
         <v>2896.1979999999999</v>
       </c>
-      <c r="T19" s="42">
+      <c r="T19" s="41">
         <v>3012.0320000000002</v>
       </c>
-      <c r="U19" s="42">
+      <c r="U19" s="41">
         <f>SUM(U7:U18)</f>
         <v>3201.4999999999995</v>
       </c>
-      <c r="V19" s="42">
+      <c r="V19" s="41">
         <f>SUM(V7:V18)</f>
         <v>3656.08</v>
       </c>
-      <c r="W19" s="42">
+      <c r="W19" s="41">
         <f>SUM(W7:W18)</f>
         <v>3619.5400000000004</v>
       </c>
-      <c r="X19" s="42">
+      <c r="X19" s="41">
         <v>3724.726000000001</v>
       </c>
-      <c r="Y19" s="42">
+      <c r="Y19" s="41">
         <f>SUM(Y7:Y18)</f>
         <v>3792.8569999999991</v>
       </c>
     </row>
     <row r="20" spans="1:25">
-      <c r="A20" s="44"/>
-      <c r="B20" s="44"/>
-      <c r="C20" s="44"/>
-      <c r="D20" s="44"/>
-      <c r="E20" s="45"/>
-      <c r="F20" s="44"/>
-      <c r="G20" s="44"/>
-      <c r="H20" s="44"/>
-      <c r="I20" s="44"/>
-      <c r="J20" s="44"/>
-      <c r="K20" s="44"/>
-      <c r="L20" s="44"/>
-      <c r="M20" s="44"/>
-      <c r="N20" s="44"/>
-      <c r="O20" s="44"/>
-      <c r="T20" s="46"/>
-      <c r="U20" s="46"/>
+      <c r="A20" s="43"/>
+      <c r="B20" s="43"/>
+      <c r="C20" s="43"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="44"/>
+      <c r="F20" s="43"/>
+      <c r="G20" s="43"/>
+      <c r="H20" s="43"/>
+      <c r="I20" s="43"/>
+      <c r="J20" s="43"/>
+      <c r="K20" s="43"/>
+      <c r="L20" s="43"/>
+      <c r="M20" s="43"/>
+      <c r="N20" s="43"/>
+      <c r="O20" s="43"/>
+      <c r="T20" s="45"/>
+      <c r="U20" s="45"/>
     </row>
     <row r="21" spans="1:25">
-      <c r="A21" s="48" t="s">
+      <c r="A21" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="T21" s="46"/>
+      <c r="T21" s="45"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>